<commit_message>
R3 = 255k e 2,2 uF su CF4/CF7/CF9 (datasheet LT3461, LP2985, MCP1825), nota per la verifica INFN
- R3 270k -> 255k: VOUT40 da 41,7 a 39,4 V, sotto i 40 V max assoluti del LT3461;
  bias ancora regolabile fino a ~39,2 V (margine 1,0 V a 25 C, 0,3 V a 50 C).
- CF4, CF7, CF9 100n -> 2,2 uF X7R 0805 (Samsung CL21B225KAFNNNE): uscite dei
  regolatori, come richiesto dai datasheet.
- Schemi, PCB (valori), BOM, file JLCPCB, PDF, simulazioni e render rigenerati;
  verifica_ltspice: tutto OK; sim_3canali invariata salvo VOUT40.
- hardware/variante_3ch/NOTA_PER_TECNICO_INFN.txt: le due modifiche con calcoli,
  simulazioni e punti da verificare, piu' l'elenco delle differenze dalla scheda INFN.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_017fc9yPsNewCQrMK8R1c8Ls
</commit_message>
<xml_diff>
--- a/hardware/bom/BOM_riv_cosmici.xlsx
+++ b/hardware/bom/BOM_riv_cosmici.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F48"/>
+  <dimension ref="A1:F49"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -544,11 +544,11 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>C4 CF1 CF2 CF3 CF4 CF5 CF6 CF7 CF8 CF9 CF10</t>
+          <t>C4 CF1 CF2 CF3 CF5 CF6 CF8 CF10</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>11</v>
+        <v>8</v>
       </c>
       <c r="C7" t="inlineStr">
         <is>
@@ -680,33 +680,33 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>D1</t>
+          <t>CF4 CF7 CF9</t>
         </is>
       </c>
       <c r="B13" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>1N4148</t>
+          <t>2.2uF</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>DO-35</t>
+          <t>0805</t>
         </is>
       </c>
       <c r="E13" t="inlineStr"/>
       <c r="F13" t="inlineStr">
         <is>
-          <t>assiale DO-35 (o 1N4148W SOD-123 adattando il footprint)</t>
+          <t>X7R 0805 &gt;= 10 V, es. Samsung CL21B225KAFNNNE (uscite regolatori; INFN: 100n)</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>D3</t>
+          <t>D1</t>
         </is>
       </c>
       <c r="B14" t="n">
@@ -714,25 +714,25 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>LED rosso</t>
+          <t>1N4148</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>0805</t>
+          <t>DO-35</t>
         </is>
       </c>
       <c r="E14" t="inlineStr"/>
       <c r="F14" t="inlineStr">
         <is>
-          <t>LED rosso 0805 (pin 1 = catodo)</t>
+          <t>assiale DO-35 (o 1N4148W SOD-123 adattando il footprint)</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>J1</t>
+          <t>D3</t>
         </is>
       </c>
       <c r="B15" t="n">
@@ -740,25 +740,25 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>SiPM</t>
+          <t>LED rosso</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>Header 2.54 1x2</t>
+          <t>0805</t>
         </is>
       </c>
       <c r="E15" t="inlineStr"/>
       <c r="F15" t="inlineStr">
         <is>
-          <t>verso scintillatore, cavo Fileca schermato; calza = bias 38,4V</t>
+          <t>LED rosso 0805 (pin 1 = catodo)</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>J2</t>
+          <t>J1</t>
         </is>
       </c>
       <c r="B16" t="n">
@@ -766,7 +766,7 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>TTL_OUT</t>
+          <t>SiPM</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
@@ -777,14 +777,14 @@
       <c r="E16" t="inlineStr"/>
       <c r="F16" t="inlineStr">
         <is>
-          <t>uscita 0-5 V (MCP1402): NON collegare ai GPIO del Raspberry Pi</t>
+          <t>verso scintillatore, cavo Fileca schermato; calza = bias 38,4V</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>J3</t>
+          <t>J2</t>
         </is>
       </c>
       <c r="B17" t="n">
@@ -792,7 +792,7 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>PWR_5V</t>
+          <t>TTL_OUT</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
@@ -803,14 +803,14 @@
       <c r="E17" t="inlineStr"/>
       <c r="F17" t="inlineStr">
         <is>
-          <t>pin 1 = GND, pin 2 = +5V</t>
+          <t>uscita 0-5 V (MCP1402): NON collegare ai GPIO del Raspberry Pi</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>J4</t>
+          <t>J3</t>
         </is>
       </c>
       <c r="B18" t="n">
@@ -818,7 +818,7 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>LEMO_OUT</t>
+          <t>PWR_5V</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
@@ -829,14 +829,14 @@
       <c r="E18" t="inlineStr"/>
       <c r="F18" t="inlineStr">
         <is>
-          <t>uscita 0-3,3 V per GPIO Raspberry Pi; footprint header 2.54 -&gt; LEMO a pannello via cavo</t>
+          <t>pin 1 = GND, pin 2 = +5V</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>L1</t>
+          <t>J4</t>
         </is>
       </c>
       <c r="B19" t="n">
@@ -844,29 +844,25 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>47uH</t>
+          <t>LEMO_OUT</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>SMD 5x5/6x6</t>
-        </is>
-      </c>
-      <c r="E19" t="inlineStr">
-        <is>
-          <t>RS 693-4344</t>
-        </is>
-      </c>
+          <t>Header 2.54 1x2</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr"/>
       <c r="F19" t="inlineStr">
         <is>
-          <t>verificare l'ingombro della parte RS effettiva contro il footprint 5x5</t>
+          <t>uscita 0-3,3 V per GPIO Raspberry Pi; footprint header 2.54 -&gt; LEMO a pannello via cavo</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Q1</t>
+          <t>L1</t>
         </is>
       </c>
       <c r="B20" t="n">
@@ -874,25 +870,29 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>BFR93A</t>
+          <t>47uH</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>SOT-23</t>
+          <t>SMD 5x5/6x6</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>RS 892-2365</t>
-        </is>
-      </c>
-      <c r="F20" t="inlineStr"/>
+          <t>RS 693-4344</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>verificare l'ingombro della parte RS effettiva contro il footprint 5x5</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Q2</t>
+          <t>Q1</t>
         </is>
       </c>
       <c r="B21" t="n">
@@ -900,7 +900,7 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>MMBTH81</t>
+          <t>BFR93A</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
@@ -910,7 +910,7 @@
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>RS 104-1196</t>
+          <t>RS 892-2365</t>
         </is>
       </c>
       <c r="F21" t="inlineStr"/>
@@ -918,37 +918,41 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>R1 R10</t>
+          <t>Q2</t>
         </is>
       </c>
       <c r="B22" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>10k</t>
+          <t>MMBTH81</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>0805</t>
-        </is>
-      </c>
-      <c r="E22" t="inlineStr"/>
+          <t>SOT-23</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>RS 104-1196</t>
+        </is>
+      </c>
       <c r="F22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>R2</t>
+          <t>R1 R10</t>
         </is>
       </c>
       <c r="B23" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>68k</t>
+          <t>10k</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
@@ -962,7 +966,7 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>R3</t>
+          <t>R2</t>
         </is>
       </c>
       <c r="B24" t="n">
@@ -970,7 +974,7 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>270k</t>
+          <t>68k</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
@@ -984,7 +988,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>R4</t>
+          <t>R3</t>
         </is>
       </c>
       <c r="B25" t="n">
@@ -992,7 +996,7 @@
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>1k2</t>
+          <t>255k</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
@@ -1001,12 +1005,16 @@
         </is>
       </c>
       <c r="E25" t="inlineStr"/>
-      <c r="F25" t="inlineStr"/>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>1% (INFN: 270k): VOUT40 39,4 V, sotto i 40 V max del LT3461</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>R5</t>
+          <t>R4</t>
         </is>
       </c>
       <c r="B26" t="n">
@@ -1014,7 +1022,7 @@
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>15k</t>
+          <t>1k2</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
@@ -1028,15 +1036,15 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>R6 R20</t>
+          <t>R5</t>
         </is>
       </c>
       <c r="B27" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>100k</t>
+          <t>15k</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
@@ -1050,15 +1058,15 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>R7</t>
+          <t>R6 R20</t>
         </is>
       </c>
       <c r="B28" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>27k</t>
+          <t>100k</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
@@ -1072,15 +1080,15 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>R8 R12 R14 R15 R16</t>
+          <t>R7</t>
         </is>
       </c>
       <c r="B29" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>1k</t>
+          <t>27k</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
@@ -1094,15 +1102,15 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>R9</t>
+          <t>R8 R12 R14 R15 R16</t>
         </is>
       </c>
       <c r="B30" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>1k8</t>
+          <t>1k</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
@@ -1116,7 +1124,7 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>R11</t>
+          <t>R9</t>
         </is>
       </c>
       <c r="B31" t="n">
@@ -1124,7 +1132,7 @@
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>5k6</t>
+          <t>1k8</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
@@ -1138,7 +1146,7 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>R13</t>
+          <t>R11</t>
         </is>
       </c>
       <c r="B32" t="n">
@@ -1146,7 +1154,7 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>560R</t>
+          <t>5k6</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
@@ -1160,7 +1168,7 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>R17</t>
+          <t>R13</t>
         </is>
       </c>
       <c r="B33" t="n">
@@ -1168,7 +1176,7 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>470R</t>
+          <t>560R</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
@@ -1182,7 +1190,7 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>R18</t>
+          <t>R17</t>
         </is>
       </c>
       <c r="B34" t="n">
@@ -1190,7 +1198,7 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>10R</t>
+          <t>470R</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
@@ -1204,7 +1212,7 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>R19</t>
+          <t>R18</t>
         </is>
       </c>
       <c r="B35" t="n">
@@ -1212,7 +1220,7 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>18k</t>
+          <t>10R</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
@@ -1226,7 +1234,7 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>R21</t>
+          <t>R19</t>
         </is>
       </c>
       <c r="B36" t="n">
@@ -1234,7 +1242,7 @@
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>82R</t>
+          <t>18k</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
@@ -1248,7 +1256,7 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>R22</t>
+          <t>R21</t>
         </is>
       </c>
       <c r="B37" t="n">
@@ -1256,7 +1264,7 @@
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>220k</t>
+          <t>82R</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
@@ -1270,7 +1278,7 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>R23</t>
+          <t>R22</t>
         </is>
       </c>
       <c r="B38" t="n">
@@ -1278,7 +1286,7 @@
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>33R</t>
+          <t>220k</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
@@ -1287,16 +1295,12 @@
         </is>
       </c>
       <c r="E38" t="inlineStr"/>
-      <c r="F38" t="inlineStr">
-        <is>
-          <t>terminazione serie del cavo verso Raspberry Pi</t>
-        </is>
-      </c>
+      <c r="F38" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>U1</t>
+          <t>R23</t>
         </is>
       </c>
       <c r="B39" t="n">
@@ -1304,25 +1308,25 @@
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>LT3461</t>
+          <t>33R</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>SOT-23-6 (ThinSOT)</t>
-        </is>
-      </c>
-      <c r="E39" t="inlineStr">
-        <is>
-          <t>Farnell 4024725</t>
-        </is>
-      </c>
-      <c r="F39" t="inlineStr"/>
+          <t>0805</t>
+        </is>
+      </c>
+      <c r="E39" t="inlineStr"/>
+      <c r="F39" t="inlineStr">
+        <is>
+          <t>terminazione serie del cavo verso Raspberry Pi</t>
+        </is>
+      </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>U2</t>
+          <t>U1</t>
         </is>
       </c>
       <c r="B40" t="n">
@@ -1330,17 +1334,17 @@
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>TLC555/LMC555</t>
+          <t>LT3461</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>SO-8</t>
+          <t>SOT-23-6 (ThinSOT)</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>RS 196-2112 (LMC555CM)</t>
+          <t>Farnell 4024725</t>
         </is>
       </c>
       <c r="F40" t="inlineStr"/>
@@ -1348,7 +1352,7 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>U3</t>
+          <t>U2</t>
         </is>
       </c>
       <c r="B41" t="n">
@@ -1356,7 +1360,7 @@
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>MAX961</t>
+          <t>TLC555/LMC555</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
@@ -1366,7 +1370,7 @@
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>RS 189-9176</t>
+          <t>RS 196-2112 (LMC555CM)</t>
         </is>
       </c>
       <c r="F41" t="inlineStr"/>
@@ -1374,7 +1378,7 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>U4</t>
+          <t>U3</t>
         </is>
       </c>
       <c r="B42" t="n">
@@ -1382,17 +1386,17 @@
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>MCP1402</t>
+          <t>MAX961</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>SOT-23-5</t>
+          <t>SO-8</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>RS 668-4203</t>
+          <t>RS 189-9176</t>
         </is>
       </c>
       <c r="F42" t="inlineStr"/>
@@ -1400,15 +1404,15 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>U5 U7</t>
+          <t>U4</t>
         </is>
       </c>
       <c r="B43" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>LP2985AIM5-3.6</t>
+          <t>MCP1402</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
@@ -1418,7 +1422,7 @@
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>RS 812-2417</t>
+          <t>RS 668-4203</t>
         </is>
       </c>
       <c r="F43" t="inlineStr"/>
@@ -1426,25 +1430,25 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>U6</t>
+          <t>U5 U7</t>
         </is>
       </c>
       <c r="B44" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>MCP1825S-3302</t>
+          <t>LP2985AIM5-3.6</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>SOT-223</t>
+          <t>SOT-23-5</t>
         </is>
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>RS 669-5092</t>
+          <t>RS 812-2417</t>
         </is>
       </c>
       <c r="F44" t="inlineStr"/>
@@ -1452,7 +1456,7 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>U8</t>
+          <t>U6</t>
         </is>
       </c>
       <c r="B45" t="n">
@@ -1460,17 +1464,17 @@
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>LT1636</t>
+          <t>MCP1825S-3302</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>SO-8</t>
+          <t>SOT-223</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>Farnell 4020771</t>
+          <t>RS 669-5092</t>
         </is>
       </c>
       <c r="F45" t="inlineStr"/>
@@ -1478,7 +1482,7 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>U9</t>
+          <t>U8</t>
         </is>
       </c>
       <c r="B46" t="n">
@@ -1486,72 +1490,98 @@
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>74LVC1G17</t>
+          <t>LT1636</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>SOT-23-5</t>
-        </is>
-      </c>
-      <c r="E46" t="inlineStr"/>
-      <c r="F46" t="inlineStr">
-        <is>
-          <t>SN74LVC1G17DBVR (TI) o equivalente; buffer 3,3 V verso Raspberry Pi</t>
-        </is>
-      </c>
+          <t>SO-8</t>
+        </is>
+      </c>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>Farnell 4020771</t>
+        </is>
+      </c>
+      <c r="F46" t="inlineStr"/>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>V1 V2</t>
+          <t>U9</t>
         </is>
       </c>
       <c r="B47" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>10k</t>
+          <t>74LVC1G17</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>Trimmer 3296W</t>
+          <t>SOT-23-5</t>
         </is>
       </c>
       <c r="E47" t="inlineStr"/>
       <c r="F47" t="inlineStr">
         <is>
-          <t>Bourns 3296W-1-103LF o equivalente</t>
+          <t>SN74LVC1G17DBVR (TI) o equivalente; buffer 3,3 V verso Raspberry Pi</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
+          <t>V1 V2</t>
+        </is>
+      </c>
+      <c r="B48" t="n">
+        <v>2</v>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>10k</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>Trimmer 3296W</t>
+        </is>
+      </c>
+      <c r="E48" t="inlineStr"/>
+      <c r="F48" t="inlineStr">
+        <is>
+          <t>Bourns 3296W-1-103LF o equivalente</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
           <t>(fuori scheda)</t>
         </is>
       </c>
-      <c r="B48" t="n">
-        <v>1</v>
-      </c>
-      <c r="C48" t="inlineStr">
+      <c r="B49" t="n">
+        <v>1</v>
+      </c>
+      <c r="C49" t="inlineStr">
         <is>
           <t>SiPM AFBR-S4N22P014M</t>
         </is>
       </c>
-      <c r="D48" t="inlineStr">
+      <c r="D49" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="E48" t="inlineStr">
+      <c r="E49" t="inlineStr">
         <is>
           <t>Farnell 4351470</t>
         </is>
       </c>
-      <c r="F48" t="inlineStr">
+      <c r="F49" t="inlineStr">
         <is>
           <t>montato su PCB separato incollato allo scintillatore</t>
         </is>

</xml_diff>